<commit_message>
feat: add EPF and ESIC fields to payroll module and update related components
</commit_message>
<xml_diff>
--- a/public/payroll-upload-sample.xlsx
+++ b/public/payroll-upload-sample.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -438,6 +438,12 @@
       <c r="L1" t="str">
         <v>Health Insurance</v>
       </c>
+      <c r="M1" t="str">
+        <v>EPF</v>
+      </c>
+      <c r="N1" t="str">
+        <v>ESIC</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -476,6 +482,12 @@
       <c r="L2">
         <v>0</v>
       </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -514,10 +526,16 @@
       <c r="L3">
         <v>300</v>
       </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>